<commit_message>
Daily recap, matchup updates, learning and research 2026-08-26
</commit_message>
<xml_diff>
--- a/data/k-props/2026-08-26.xlsx
+++ b/data/k-props/2026-08-26.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="100">
   <si>
     <t>date</t>
   </si>
@@ -145,6 +145,9 @@
     <t>lineup_unweighted_30d_posted</t>
   </si>
   <si>
+    <t>U</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
@@ -154,6 +157,9 @@
     <t>Troy Melton</t>
   </si>
   <si>
+    <t>O</t>
+  </si>
+  <si>
     <t>Matthew Boyd</t>
   </si>
   <si>
@@ -184,6 +190,9 @@
     <t>Grayson Rodriguez</t>
   </si>
   <si>
+    <t>W</t>
+  </si>
+  <si>
     <t>Bubba Chandler</t>
   </si>
   <si>
@@ -233,6 +242,9 @@
   </si>
   <si>
     <t>Elmer Rodríguez</t>
+  </si>
+  <si>
+    <t>L</t>
   </si>
   <si>
     <t>Randy Dobnak</t>
@@ -880,17 +892,23 @@
       <c r="Y2">
         <v>0.9046</v>
       </c>
+      <c r="Z2">
+        <v>4</v>
+      </c>
       <c r="AA2" t="s">
         <v>44</v>
       </c>
+      <c r="AB2">
+        <v>-0.66</v>
+      </c>
       <c r="AC2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD2">
         <v>3.64</v>
       </c>
       <c r="AE2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF2">
         <v>0.2033</v>
@@ -900,6 +918,18 @@
       </c>
       <c r="AH2">
         <v>0.2</v>
+      </c>
+      <c r="AI2">
+        <v>0.36</v>
+      </c>
+      <c r="AJ2">
+        <v>0.36</v>
+      </c>
+      <c r="AK2">
+        <v>0.16</v>
+      </c>
+      <c r="AL2">
+        <v>0.16</v>
       </c>
       <c r="AM2">
         <v>3.84</v>
@@ -910,7 +940,7 @@
         <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C3">
         <v>3.5</v>
@@ -981,17 +1011,23 @@
       <c r="Y3">
         <v>0.88</v>
       </c>
+      <c r="Z3">
+        <v>4</v>
+      </c>
       <c r="AA3" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB3">
+        <v>-0.47</v>
       </c>
       <c r="AC3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD3">
         <v>2.83</v>
       </c>
       <c r="AE3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF3">
         <v>0.1922</v>
@@ -1001,6 +1037,18 @@
       </c>
       <c r="AH3">
         <v>0.2</v>
+      </c>
+      <c r="AI3">
+        <v>1.17</v>
+      </c>
+      <c r="AJ3">
+        <v>1.17</v>
+      </c>
+      <c r="AK3">
+        <v>0.97</v>
+      </c>
+      <c r="AL3">
+        <v>0.97</v>
       </c>
       <c r="AM3">
         <v>3.03</v>
@@ -1011,7 +1059,7 @@
         <v>39</v>
       </c>
       <c r="B4" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="C4">
         <v>3.5</v>
@@ -1023,7 +1071,7 @@
         <v>105</v>
       </c>
       <c r="F4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G4">
         <v>825039</v>
@@ -1082,17 +1130,23 @@
       <c r="Y4">
         <v>0.88</v>
       </c>
+      <c r="Z4">
+        <v>5</v>
+      </c>
       <c r="AA4" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB4">
+        <v>-0.31</v>
       </c>
       <c r="AC4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD4">
         <v>2.99</v>
       </c>
       <c r="AE4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF4">
         <v>0.1648</v>
@@ -1102,6 +1156,18 @@
       </c>
       <c r="AH4">
         <v>0.2</v>
+      </c>
+      <c r="AI4">
+        <v>2.01</v>
+      </c>
+      <c r="AJ4">
+        <v>2.01</v>
+      </c>
+      <c r="AK4">
+        <v>1.81</v>
+      </c>
+      <c r="AL4">
+        <v>1.81</v>
       </c>
       <c r="AM4">
         <v>3.19</v>
@@ -1112,7 +1178,7 @@
         <v>39</v>
       </c>
       <c r="B5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="C5">
         <v>4.5</v>
@@ -1124,7 +1190,7 @@
         <v>-155</v>
       </c>
       <c r="F5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G5">
         <v>825039</v>
@@ -1183,17 +1249,23 @@
       <c r="Y5">
         <v>0.8982</v>
       </c>
+      <c r="Z5">
+        <v>9</v>
+      </c>
       <c r="AA5" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB5">
+        <v>-0.18</v>
       </c>
       <c r="AC5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD5">
         <v>4.12</v>
       </c>
       <c r="AE5" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF5">
         <v>0.2043</v>
@@ -1203,6 +1275,18 @@
       </c>
       <c r="AH5">
         <v>0.2</v>
+      </c>
+      <c r="AI5">
+        <v>4.88</v>
+      </c>
+      <c r="AJ5">
+        <v>4.88</v>
+      </c>
+      <c r="AK5">
+        <v>4.68</v>
+      </c>
+      <c r="AL5">
+        <v>4.68</v>
       </c>
       <c r="AM5">
         <v>4.32</v>
@@ -1213,7 +1297,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C6">
         <v>4.5</v>
@@ -1225,7 +1309,7 @@
         <v>111</v>
       </c>
       <c r="F6" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G6">
         <v>823180</v>
@@ -1284,17 +1368,23 @@
       <c r="Y6">
         <v>0.9287</v>
       </c>
+      <c r="Z6">
+        <v>5</v>
+      </c>
       <c r="AA6" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB6">
+        <v>0.04</v>
       </c>
       <c r="AC6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD6">
         <v>4.34</v>
       </c>
       <c r="AE6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF6">
         <v>0.1777</v>
@@ -1304,6 +1394,18 @@
       </c>
       <c r="AH6">
         <v>0.2</v>
+      </c>
+      <c r="AI6">
+        <v>0.66</v>
+      </c>
+      <c r="AJ6">
+        <v>0.66</v>
+      </c>
+      <c r="AK6">
+        <v>0.46</v>
+      </c>
+      <c r="AL6">
+        <v>0.46</v>
       </c>
       <c r="AM6">
         <v>4.54</v>
@@ -1314,7 +1416,7 @@
         <v>39</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7">
         <v>5.5</v>
@@ -1326,7 +1428,7 @@
         <v>117</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G7">
         <v>823180</v>
@@ -1385,17 +1487,23 @@
       <c r="Y7">
         <v>1.0648</v>
       </c>
+      <c r="Z7">
+        <v>6</v>
+      </c>
       <c r="AA7" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB7">
+        <v>0.64</v>
       </c>
       <c r="AC7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD7">
         <v>6.35</v>
       </c>
       <c r="AE7" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF7">
         <v>0.2023</v>
@@ -1405,6 +1513,18 @@
       </c>
       <c r="AH7">
         <v>-0.21</v>
+      </c>
+      <c r="AI7">
+        <v>-0.35</v>
+      </c>
+      <c r="AJ7">
+        <v>0.35</v>
+      </c>
+      <c r="AK7">
+        <v>-0.14</v>
+      </c>
+      <c r="AL7">
+        <v>0.14</v>
       </c>
       <c r="AM7">
         <v>6.14</v>
@@ -1415,7 +1535,7 @@
         <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C8">
         <v>6.5</v>
@@ -1427,7 +1547,7 @@
         <v>110</v>
       </c>
       <c r="F8" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G8">
         <v>823988</v>
@@ -1486,17 +1606,23 @@
       <c r="Y8">
         <v>1.0973</v>
       </c>
+      <c r="Z8">
+        <v>1</v>
+      </c>
       <c r="AA8" t="s">
         <v>44</v>
       </c>
+      <c r="AB8">
+        <v>-0.02</v>
+      </c>
       <c r="AC8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD8">
         <v>6.69</v>
       </c>
       <c r="AE8" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF8">
         <v>0.2365</v>
@@ -1506,6 +1632,18 @@
       </c>
       <c r="AH8">
         <v>-0.21</v>
+      </c>
+      <c r="AI8">
+        <v>-5.69</v>
+      </c>
+      <c r="AJ8">
+        <v>5.69</v>
+      </c>
+      <c r="AK8">
+        <v>-5.48</v>
+      </c>
+      <c r="AL8">
+        <v>5.48</v>
       </c>
       <c r="AM8">
         <v>6.48</v>
@@ -1516,7 +1654,7 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C9">
         <v>4.5</v>
@@ -1528,7 +1666,7 @@
         <v>-156</v>
       </c>
       <c r="F9" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G9">
         <v>823988</v>
@@ -1587,17 +1725,23 @@
       <c r="Y9">
         <v>0.88</v>
       </c>
+      <c r="Z9">
+        <v>4</v>
+      </c>
       <c r="AA9" t="s">
         <v>44</v>
       </c>
+      <c r="AB9">
+        <v>-0.95</v>
+      </c>
       <c r="AC9" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="AD9">
         <v>3.35</v>
       </c>
       <c r="AE9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF9">
         <v>0.2209</v>
@@ -1607,6 +1751,18 @@
       </c>
       <c r="AH9">
         <v>0.2</v>
+      </c>
+      <c r="AI9">
+        <v>0.65</v>
+      </c>
+      <c r="AJ9">
+        <v>0.65</v>
+      </c>
+      <c r="AK9">
+        <v>0.45</v>
+      </c>
+      <c r="AL9">
+        <v>0.45</v>
       </c>
       <c r="AM9">
         <v>3.55</v>
@@ -1617,7 +1773,7 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C10">
         <v>4.5</v>
@@ -1629,7 +1785,7 @@
         <v>-147</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G10">
         <v>823255</v>
@@ -1688,17 +1844,23 @@
       <c r="Y10">
         <v>1.002</v>
       </c>
+      <c r="Z10">
+        <v>3</v>
+      </c>
       <c r="AA10" t="s">
         <v>44</v>
       </c>
+      <c r="AB10">
+        <v>-0.32</v>
+      </c>
       <c r="AC10" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD10">
         <v>3.98</v>
       </c>
       <c r="AE10" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF10">
         <v>0.2128</v>
@@ -1708,6 +1870,18 @@
       </c>
       <c r="AH10">
         <v>0.2</v>
+      </c>
+      <c r="AI10">
+        <v>-0.98</v>
+      </c>
+      <c r="AJ10">
+        <v>0.98</v>
+      </c>
+      <c r="AK10">
+        <v>-1.18</v>
+      </c>
+      <c r="AL10">
+        <v>1.18</v>
       </c>
       <c r="AM10">
         <v>4.18</v>
@@ -1718,7 +1892,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C11">
         <v>3.5</v>
@@ -1730,7 +1904,7 @@
         <v>-119</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="G11">
         <v>823255</v>
@@ -1789,17 +1963,23 @@
       <c r="Y11">
         <v>1.0872</v>
       </c>
+      <c r="Z11">
+        <v>2</v>
+      </c>
       <c r="AA11" t="s">
         <v>44</v>
       </c>
+      <c r="AB11">
+        <v>0.4</v>
+      </c>
       <c r="AC11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD11">
         <v>3.7</v>
       </c>
       <c r="AE11" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF11">
         <v>0.1262</v>
@@ -1809,6 +1989,18 @@
       </c>
       <c r="AH11">
         <v>0.2</v>
+      </c>
+      <c r="AI11">
+        <v>-1.7</v>
+      </c>
+      <c r="AJ11">
+        <v>1.7</v>
+      </c>
+      <c r="AK11">
+        <v>-1.9</v>
+      </c>
+      <c r="AL11">
+        <v>1.9</v>
       </c>
       <c r="AM11">
         <v>3.9</v>
@@ -1819,7 +2011,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C12">
         <v>7.5</v>
@@ -1831,7 +2023,7 @@
         <v>-105</v>
       </c>
       <c r="F12" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G12">
         <v>823096</v>
@@ -1890,17 +2082,23 @@
       <c r="Y12">
         <v>0.926</v>
       </c>
+      <c r="Z12">
+        <v>9</v>
+      </c>
       <c r="AA12" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB12">
+        <v>1.34</v>
       </c>
       <c r="AC12" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="AD12">
         <v>9.75</v>
       </c>
       <c r="AE12" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AF12">
         <v>0.3201</v>
@@ -1910,6 +2108,18 @@
       </c>
       <c r="AH12">
         <v>-0.91</v>
+      </c>
+      <c r="AI12">
+        <v>-0.75</v>
+      </c>
+      <c r="AJ12">
+        <v>0.75</v>
+      </c>
+      <c r="AK12">
+        <v>0.16</v>
+      </c>
+      <c r="AL12">
+        <v>0.16</v>
       </c>
       <c r="AM12">
         <v>8.84</v>
@@ -1920,7 +2130,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C13">
         <v>5.5</v>
@@ -1932,7 +2142,7 @@
         <v>-153</v>
       </c>
       <c r="F13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="G13">
         <v>823096</v>
@@ -1991,17 +2201,23 @@
       <c r="Y13">
         <v>0.9267</v>
       </c>
+      <c r="Z13">
+        <v>5</v>
+      </c>
       <c r="AA13" t="s">
         <v>44</v>
       </c>
+      <c r="AB13">
+        <v>-1.55</v>
+      </c>
       <c r="AC13" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="AD13">
         <v>3.75</v>
       </c>
       <c r="AE13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF13">
         <v>0.2512</v>
@@ -2011,6 +2227,18 @@
       </c>
       <c r="AH13">
         <v>0.2</v>
+      </c>
+      <c r="AI13">
+        <v>1.25</v>
+      </c>
+      <c r="AJ13">
+        <v>1.25</v>
+      </c>
+      <c r="AK13">
+        <v>1.05</v>
+      </c>
+      <c r="AL13">
+        <v>1.05</v>
       </c>
       <c r="AM13">
         <v>3.95</v>
@@ -2021,7 +2249,7 @@
         <v>39</v>
       </c>
       <c r="B14" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C14">
         <v>5.5</v>
@@ -2033,7 +2261,7 @@
         <v>100</v>
       </c>
       <c r="F14" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G14">
         <v>823825</v>
@@ -2092,17 +2320,23 @@
       <c r="Y14">
         <v>0.9306</v>
       </c>
+      <c r="Z14">
+        <v>5</v>
+      </c>
       <c r="AA14" t="s">
         <v>44</v>
       </c>
+      <c r="AB14">
+        <v>-0.67</v>
+      </c>
       <c r="AC14" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD14">
         <v>4.63</v>
       </c>
       <c r="AE14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF14">
         <v>0.222</v>
@@ -2112,6 +2346,18 @@
       </c>
       <c r="AH14">
         <v>0.2</v>
+      </c>
+      <c r="AI14">
+        <v>0.37</v>
+      </c>
+      <c r="AJ14">
+        <v>0.37</v>
+      </c>
+      <c r="AK14">
+        <v>0.17</v>
+      </c>
+      <c r="AL14">
+        <v>0.17</v>
       </c>
       <c r="AM14">
         <v>4.83</v>
@@ -2122,7 +2368,7 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C15">
         <v>3.5</v>
@@ -2134,13 +2380,13 @@
         <v>117</v>
       </c>
       <c r="F15" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="G15">
         <v>823825</v>
       </c>
       <c r="H15" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I15">
         <v>4</v>
@@ -2193,17 +2439,23 @@
       <c r="Y15">
         <v>0.9774</v>
       </c>
+      <c r="Z15">
+        <v>2</v>
+      </c>
       <c r="AA15" t="s">
         <v>44</v>
       </c>
+      <c r="AB15">
+        <v>-0.76</v>
+      </c>
       <c r="AC15" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="AD15">
         <v>2.54</v>
       </c>
       <c r="AE15" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF15">
         <v>0.1974</v>
@@ -2213,6 +2465,18 @@
       </c>
       <c r="AH15">
         <v>0.2</v>
+      </c>
+      <c r="AI15">
+        <v>-0.54</v>
+      </c>
+      <c r="AJ15">
+        <v>0.54</v>
+      </c>
+      <c r="AK15">
+        <v>-0.74</v>
+      </c>
+      <c r="AL15">
+        <v>0.74</v>
       </c>
       <c r="AM15">
         <v>2.74</v>
@@ -2223,7 +2487,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C16">
         <v>3.5</v>
@@ -2235,7 +2499,7 @@
         <v>-103</v>
       </c>
       <c r="F16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G16">
         <v>822692</v>
@@ -2294,17 +2558,23 @@
       <c r="Y16">
         <v>1.0422</v>
       </c>
+      <c r="Z16">
+        <v>5</v>
+      </c>
       <c r="AA16" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB16">
+        <v>0.76</v>
       </c>
       <c r="AC16" t="s">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="AD16">
         <v>4.06</v>
       </c>
       <c r="AE16" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF16">
         <v>0.1721</v>
@@ -2314,6 +2584,18 @@
       </c>
       <c r="AH16">
         <v>0.2</v>
+      </c>
+      <c r="AI16">
+        <v>0.94</v>
+      </c>
+      <c r="AJ16">
+        <v>0.94</v>
+      </c>
+      <c r="AK16">
+        <v>0.74</v>
+      </c>
+      <c r="AL16">
+        <v>0.74</v>
       </c>
       <c r="AM16">
         <v>4.26</v>
@@ -2324,10 +2606,10 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="F17" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G17">
         <v>822692</v>
@@ -2387,16 +2669,16 @@
         <v>1.0263</v>
       </c>
       <c r="AA17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC17" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD17">
         <v>3.91</v>
       </c>
       <c r="AE17" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF17">
         <v>0.1661</v>
@@ -2416,7 +2698,7 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C18">
         <v>5.5</v>
@@ -2428,7 +2710,7 @@
         <v>-142</v>
       </c>
       <c r="F18" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G18">
         <v>823506</v>
@@ -2487,17 +2769,23 @@
       <c r="Y18">
         <v>0.9712</v>
       </c>
+      <c r="Z18">
+        <v>5</v>
+      </c>
       <c r="AA18" t="s">
         <v>44</v>
       </c>
+      <c r="AB18">
+        <v>0.4</v>
+      </c>
       <c r="AC18" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD18">
         <v>6.11</v>
       </c>
       <c r="AE18" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF18">
         <v>0.2332</v>
@@ -2507,6 +2795,18 @@
       </c>
       <c r="AH18">
         <v>-0.21</v>
+      </c>
+      <c r="AI18">
+        <v>-1.11</v>
+      </c>
+      <c r="AJ18">
+        <v>1.11</v>
+      </c>
+      <c r="AK18">
+        <v>-0.9</v>
+      </c>
+      <c r="AL18">
+        <v>0.9</v>
       </c>
       <c r="AM18">
         <v>5.9</v>
@@ -2517,7 +2817,7 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C19">
         <v>3.5</v>
@@ -2529,13 +2829,13 @@
         <v>106</v>
       </c>
       <c r="F19" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="G19">
         <v>823506</v>
       </c>
       <c r="H19" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I19">
         <v>4.3</v>
@@ -2588,17 +2888,23 @@
       <c r="Y19">
         <v>0.9926</v>
       </c>
+      <c r="Z19">
+        <v>6</v>
+      </c>
       <c r="AA19" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB19">
+        <v>-0.82</v>
       </c>
       <c r="AC19" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="AD19">
         <v>2.48</v>
       </c>
       <c r="AE19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF19">
         <v>0.1205</v>
@@ -2608,6 +2914,18 @@
       </c>
       <c r="AH19">
         <v>0.2</v>
+      </c>
+      <c r="AI19">
+        <v>3.52</v>
+      </c>
+      <c r="AJ19">
+        <v>3.52</v>
+      </c>
+      <c r="AK19">
+        <v>3.32</v>
+      </c>
+      <c r="AL19">
+        <v>3.32</v>
       </c>
       <c r="AM19">
         <v>2.68</v>
@@ -2618,7 +2936,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="C20">
         <v>2.5</v>
@@ -2630,7 +2948,7 @@
         <v>102</v>
       </c>
       <c r="F20" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G20">
         <v>822772</v>
@@ -2689,17 +3007,23 @@
       <c r="Y20">
         <v>0.9603</v>
       </c>
+      <c r="Z20">
+        <v>5</v>
+      </c>
       <c r="AA20" t="s">
-        <v>44</v>
+        <v>48</v>
+      </c>
+      <c r="AB20">
+        <v>0.28</v>
       </c>
       <c r="AC20" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD20">
         <v>2.58</v>
       </c>
       <c r="AE20" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF20">
         <v>0.1538</v>
@@ -2709,6 +3033,18 @@
       </c>
       <c r="AH20">
         <v>0.2</v>
+      </c>
+      <c r="AI20">
+        <v>2.42</v>
+      </c>
+      <c r="AJ20">
+        <v>2.42</v>
+      </c>
+      <c r="AK20">
+        <v>2.22</v>
+      </c>
+      <c r="AL20">
+        <v>2.22</v>
       </c>
       <c r="AM20">
         <v>2.78</v>
@@ -2719,16 +3055,16 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="F21" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G21">
         <v>822772</v>
       </c>
       <c r="H21" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="I21">
         <v>3</v>
@@ -2782,16 +3118,16 @@
         <v>0.9489</v>
       </c>
       <c r="AA21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC21" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD21">
         <v>1.93</v>
       </c>
       <c r="AE21" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF21">
         <v>0.2048</v>
@@ -2811,7 +3147,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C22">
         <v>4.5</v>
@@ -2823,7 +3159,7 @@
         <v>100</v>
       </c>
       <c r="F22" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G22">
         <v>823584</v>
@@ -2882,17 +3218,23 @@
       <c r="Y22">
         <v>0.9909</v>
       </c>
+      <c r="Z22">
+        <v>0</v>
+      </c>
       <c r="AA22" t="s">
         <v>44</v>
       </c>
+      <c r="AB22">
+        <v>0.79</v>
+      </c>
       <c r="AC22" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="AD22">
         <v>5.09</v>
       </c>
       <c r="AE22" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF22">
         <v>0.2205</v>
@@ -2902,6 +3244,18 @@
       </c>
       <c r="AH22">
         <v>0.2</v>
+      </c>
+      <c r="AI22">
+        <v>-5.09</v>
+      </c>
+      <c r="AJ22">
+        <v>5.09</v>
+      </c>
+      <c r="AK22">
+        <v>-5.29</v>
+      </c>
+      <c r="AL22">
+        <v>5.29</v>
       </c>
       <c r="AM22">
         <v>5.29</v>
@@ -2912,7 +3266,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C23">
         <v>4.5</v>
@@ -2924,13 +3278,13 @@
         <v>-129</v>
       </c>
       <c r="F23" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="G23">
         <v>823584</v>
       </c>
       <c r="H23" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="I23">
         <v>4.2</v>
@@ -2983,17 +3337,23 @@
       <c r="Y23">
         <v>0.9835</v>
       </c>
+      <c r="Z23">
+        <v>2</v>
+      </c>
       <c r="AA23" t="s">
         <v>44</v>
       </c>
+      <c r="AB23">
+        <v>0.36</v>
+      </c>
       <c r="AC23" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD23">
         <v>4.66</v>
       </c>
       <c r="AE23" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF23">
         <v>0.2346</v>
@@ -3003,6 +3363,18 @@
       </c>
       <c r="AH23">
         <v>0.2</v>
+      </c>
+      <c r="AI23">
+        <v>-2.66</v>
+      </c>
+      <c r="AJ23">
+        <v>2.66</v>
+      </c>
+      <c r="AK23">
+        <v>-2.86</v>
+      </c>
+      <c r="AL23">
+        <v>2.86</v>
       </c>
       <c r="AM23">
         <v>4.86</v>
@@ -3013,7 +3385,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C24">
         <v>4.5</v>
@@ -3025,7 +3397,7 @@
         <v>128</v>
       </c>
       <c r="F24" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G24">
         <v>824878</v>
@@ -3084,17 +3456,23 @@
       <c r="Y24">
         <v>0.9998</v>
       </c>
+      <c r="Z24">
+        <v>3</v>
+      </c>
       <c r="AA24" t="s">
         <v>44</v>
       </c>
+      <c r="AB24">
+        <v>1.29</v>
+      </c>
       <c r="AC24" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="AD24">
         <v>5.59</v>
       </c>
       <c r="AE24" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF24">
         <v>0.2359</v>
@@ -3104,6 +3482,18 @@
       </c>
       <c r="AH24">
         <v>0.2</v>
+      </c>
+      <c r="AI24">
+        <v>-2.59</v>
+      </c>
+      <c r="AJ24">
+        <v>2.59</v>
+      </c>
+      <c r="AK24">
+        <v>-2.79</v>
+      </c>
+      <c r="AL24">
+        <v>2.79</v>
       </c>
       <c r="AM24">
         <v>5.79</v>
@@ -3114,7 +3504,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C25">
         <v>6.5</v>
@@ -3126,7 +3516,7 @@
         <v>-143</v>
       </c>
       <c r="F25" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G25">
         <v>824555</v>
@@ -3185,17 +3575,23 @@
       <c r="Y25">
         <v>1.0284</v>
       </c>
+      <c r="Z25">
+        <v>4</v>
+      </c>
       <c r="AA25" t="s">
         <v>44</v>
       </c>
+      <c r="AB25">
+        <v>0.17</v>
+      </c>
       <c r="AC25" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD25">
         <v>6.88</v>
       </c>
       <c r="AE25" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF25">
         <v>0.268</v>
@@ -3205,6 +3601,18 @@
       </c>
       <c r="AH25">
         <v>-0.21</v>
+      </c>
+      <c r="AI25">
+        <v>-2.88</v>
+      </c>
+      <c r="AJ25">
+        <v>2.88</v>
+      </c>
+      <c r="AK25">
+        <v>-2.67</v>
+      </c>
+      <c r="AL25">
+        <v>2.67</v>
       </c>
       <c r="AM25">
         <v>6.67</v>
@@ -3215,7 +3623,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C26">
         <v>5.5</v>
@@ -3227,7 +3635,7 @@
         <v>120</v>
       </c>
       <c r="F26" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="G26">
         <v>824555</v>
@@ -3286,17 +3694,23 @@
       <c r="Y26">
         <v>1.0558</v>
       </c>
+      <c r="Z26">
+        <v>3</v>
+      </c>
       <c r="AA26" t="s">
         <v>44</v>
       </c>
+      <c r="AB26">
+        <v>0.63</v>
+      </c>
       <c r="AC26" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD26">
         <v>6.34</v>
       </c>
       <c r="AE26" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF26">
         <v>0.258</v>
@@ -3306,6 +3720,18 @@
       </c>
       <c r="AH26">
         <v>-0.21</v>
+      </c>
+      <c r="AI26">
+        <v>-3.34</v>
+      </c>
+      <c r="AJ26">
+        <v>3.34</v>
+      </c>
+      <c r="AK26">
+        <v>-3.13</v>
+      </c>
+      <c r="AL26">
+        <v>3.13</v>
       </c>
       <c r="AM26">
         <v>6.13</v>
@@ -3316,7 +3742,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C27">
         <v>4.5</v>
@@ -3328,7 +3754,7 @@
         <v>-110</v>
       </c>
       <c r="F27" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G27">
         <v>823015</v>
@@ -3387,17 +3813,23 @@
       <c r="Y27">
         <v>0.9078</v>
       </c>
+      <c r="Z27">
+        <v>4</v>
+      </c>
       <c r="AA27" t="s">
         <v>44</v>
       </c>
+      <c r="AB27">
+        <v>0.81</v>
+      </c>
       <c r="AC27" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="AD27">
         <v>5.11</v>
       </c>
       <c r="AE27" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF27">
         <v>0.2031</v>
@@ -3407,6 +3839,18 @@
       </c>
       <c r="AH27">
         <v>0.2</v>
+      </c>
+      <c r="AI27">
+        <v>-1.11</v>
+      </c>
+      <c r="AJ27">
+        <v>1.11</v>
+      </c>
+      <c r="AK27">
+        <v>-1.31</v>
+      </c>
+      <c r="AL27">
+        <v>1.31</v>
       </c>
       <c r="AM27">
         <v>5.31</v>
@@ -3417,7 +3861,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C28">
         <v>4.5</v>
@@ -3429,7 +3873,7 @@
         <v>-137</v>
       </c>
       <c r="F28" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="G28">
         <v>823015</v>
@@ -3488,17 +3932,23 @@
       <c r="Y28">
         <v>1.0581</v>
       </c>
+      <c r="Z28">
+        <v>3</v>
+      </c>
       <c r="AA28" t="s">
         <v>44</v>
       </c>
+      <c r="AB28">
+        <v>1</v>
+      </c>
       <c r="AC28" t="s">
-        <v>44</v>
+        <v>77</v>
       </c>
       <c r="AD28">
         <v>5.3</v>
       </c>
       <c r="AE28" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF28">
         <v>0.1811</v>
@@ -3508,6 +3958,18 @@
       </c>
       <c r="AH28">
         <v>0.2</v>
+      </c>
+      <c r="AI28">
+        <v>-2.3</v>
+      </c>
+      <c r="AJ28">
+        <v>2.3</v>
+      </c>
+      <c r="AK28">
+        <v>-2.5</v>
+      </c>
+      <c r="AL28">
+        <v>2.5</v>
       </c>
       <c r="AM28">
         <v>5.5</v>
@@ -3518,7 +3980,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="C29">
         <v>5.5</v>
@@ -3530,7 +3992,7 @@
         <v>-120</v>
       </c>
       <c r="F29" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G29">
         <v>824963</v>
@@ -3589,17 +4051,23 @@
       <c r="Y29">
         <v>1.067</v>
       </c>
+      <c r="Z29">
+        <v>5</v>
+      </c>
       <c r="AA29" t="s">
         <v>44</v>
       </c>
+      <c r="AB29">
+        <v>0.45</v>
+      </c>
       <c r="AC29" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD29">
         <v>6.16</v>
       </c>
       <c r="AE29" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="AF29">
         <v>0.2532</v>
@@ -3609,6 +4077,18 @@
       </c>
       <c r="AH29">
         <v>-0.21</v>
+      </c>
+      <c r="AI29">
+        <v>-1.16</v>
+      </c>
+      <c r="AJ29">
+        <v>1.16</v>
+      </c>
+      <c r="AK29">
+        <v>-0.95</v>
+      </c>
+      <c r="AL29">
+        <v>0.95</v>
       </c>
       <c r="AM29">
         <v>5.95</v>
@@ -3619,10 +4099,10 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="F30" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G30">
         <v>824963</v>
@@ -3682,16 +4162,16 @@
         <v>0.9268</v>
       </c>
       <c r="AA30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC30" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD30">
         <v>3.67</v>
       </c>
       <c r="AE30" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AF30">
         <v>0.2104</v>
@@ -3711,7 +4191,7 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C31">
         <v>4.5</v>
@@ -3723,31 +4203,34 @@
         <v>-155</v>
       </c>
       <c r="F31" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L31">
         <v>4</v>
       </c>
       <c r="S31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V31" t="s">
-        <v>44</v>
+        <v>45</v>
+      </c>
+      <c r="Z31">
+        <v>3</v>
       </c>
       <c r="AA31" t="s">
         <v>44</v>
       </c>
       <c r="AC31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE31" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:39" x14ac:dyDescent="0.25">
@@ -3755,7 +4238,7 @@
         <v>39</v>
       </c>
       <c r="B32" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C32">
         <v>4.5</v>
@@ -3767,31 +4250,31 @@
         <v>-130</v>
       </c>
       <c r="F32" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="G32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="L32">
         <v>6</v>
       </c>
       <c r="S32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="V32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AA32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AE32" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:39" x14ac:dyDescent="0.25">
@@ -3799,7 +4282,7 @@
         <v>39</v>
       </c>
       <c r="B33" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C33">
         <v>5.5</v>
@@ -3811,7 +4294,7 @@
         <v>102</v>
       </c>
       <c r="F33" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G33">
         <v>823180</v>
@@ -3850,7 +4333,7 @@
         <v>0.369</v>
       </c>
       <c r="S33" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="T33">
         <v>0.3543</v>
@@ -3871,16 +4354,16 @@
         <v>1.0313</v>
       </c>
       <c r="AA33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AC33" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="AD33">
         <v>7.38</v>
       </c>
       <c r="AE33" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="AF33">
         <v>0.1965</v>

</xml_diff>